<commit_message>
docs(asvs): finish reconciling checklist V12–V17 with current implementation
</commit_message>
<xml_diff>
--- a/Deliverables/ASVS_5_0_Tracker.xlsx
+++ b/Deliverables/ASVS_5_0_Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\loura\Desktop\Mestrado\desofs2026_wed_ffs_3\Deliverables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F813DFFD-6E44-4504-81F1-25561B2C9B17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00DC7910-74FB-4FA6-8722-7F7B44D0A0BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" firstSheet="9" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" firstSheet="13" activeTab="16" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -2872,9 +2872,6 @@
     <t>Verify that if a credential has to be used for service authentication, the credential being used by the consumer is not a default credential (e.g., root/root or admin/admin).</t>
   </si>
   <si>
-    <t>PostgreSQL must not use default credentials (postgres/postgres)</t>
-  </si>
-  <si>
     <t>V13.2.4</t>
   </si>
   <si>
@@ -2920,9 +2917,6 @@
     <t>Verify that a secrets management solution, such as a key vault, is used to securely create, store, control access to, and destroy backend secrets. These could include passwords, key material, integrations with databases and third-party systems, keys and seeds for time-based tokens, other internal secrets, and API keys. Secrets must not be included in application source code or included in build artifacts. For an L3 application, this must involve a hardware-backed solution such as an HSM.</t>
   </si>
   <si>
-    <t>Minimum: environment variables via Docker secrets or .env file not committed to git — SDR18</t>
-  </si>
-  <si>
     <t>SDR18, SDR18a</t>
   </si>
   <si>
@@ -3001,9 +2995,6 @@
     <t>Verify that using the HTTP TRACE method is not supported in production environments, to avoid potential information leakage.</t>
   </si>
   <si>
-    <t>Must be disabled in Spring Boot / embedded Tomcat configuration</t>
-  </si>
-  <si>
     <t>SDR11</t>
   </si>
   <si>
@@ -3082,9 +3073,6 @@
     <t>Verify that sensitive data is only sent to the server in the HTTP message body or header fields, and that the URL and query string do not contain sensitive information, such as an API key or session token.</t>
   </si>
   <si>
-    <t>Gap tapado com SDR16a — passwords/tokens must never appear in URLs</t>
-  </si>
-  <si>
     <t>SDR16a</t>
   </si>
   <si>
@@ -3094,9 +3082,6 @@
     <t>Verify that the application prevents sensitive data from being cached in server components, such as load balancers and application caches, or ensures that the data is securely purged after use.</t>
   </si>
   <si>
-    <t>Gap tapado com SDR16b — Cache-Control: no-store on sensitive responses</t>
-  </si>
-  <si>
     <t>SDR16b</t>
   </si>
   <si>
@@ -3127,18 +3112,12 @@
     <t>Verify that caching mechanisms are configured to only cache responses which have the expected content type for that resource and do not contain sensitive, dynamic content. The web server should return a 404 or 302 response when a non-existent file is accessed rather than returning a different, valid file. This should prevent Web Cache Deception attacks.</t>
   </si>
   <si>
-    <t>Spring Boot responses must set explicit Content-Type; caching disabled for API endpoints</t>
-  </si>
-  <si>
     <t>V14.2.6</t>
   </si>
   <si>
     <t>Verify that the application only returns the minimum required sensitive data for the application's functionality. For example, only returning some of the digits of a credit card number and not the full number. If the complete data is required, it should be masked in the user interface unless the user specifically views it.</t>
   </si>
   <si>
-    <t>SDR09 — response serialization must exclude internal fields (password hash, internal IDs)</t>
-  </si>
-  <si>
     <t>V14.2.7</t>
   </si>
   <si>
@@ -3181,9 +3160,6 @@
     <t>Verify that the application sets sufficient anti-caching HTTP response header fields (i.e., Cache-Control: no-store) so that sensitive data is not cached in browsers.</t>
   </si>
   <si>
-    <t>Gap tapado com SDR16b — required for all sensitive endpoints</t>
-  </si>
-  <si>
     <t>V14.3.3</t>
   </si>
   <si>
@@ -3304,9 +3280,6 @@
     <t>Verify that third-party components and all of their transitive dependencies are included from the expected repository, whether internally owned or an external source, and that there is no risk of a dependency confusion attack.</t>
   </si>
   <si>
-    <t>Maven Central only; verify no unofficial repository mirrors in pom.xml</t>
-  </si>
-  <si>
     <t>SDR22, SDR22a</t>
   </si>
   <si>
@@ -3316,9 +3289,6 @@
     <t>Verify that the application implements additional protections around parts of the application which are documented as containing "dangerous functionality" or using third-party libraries considered to be "risky components". This could include techniques such as sandboxing, encapsulation, containerization or network level isolation to delay and deter attackers who compromise one part of an application from pivoting elsewhere in the application.</t>
   </si>
   <si>
-    <t>File operations (FR22/FR23) have allowlist (SDR13) + dedicated directory (SDR14)</t>
-  </si>
-  <si>
     <t>SDR13, SDR14</t>
   </si>
   <si>
@@ -3334,9 +3304,6 @@
     <t>Verify that the application only returns the required subset of fields from a data object. For example, it should not return an entire data object, as some individual fields should not be accessible to users.</t>
   </si>
   <si>
-    <t>SDR09 — response DTOs must exclude password hash, internal IDs, tokens</t>
-  </si>
-  <si>
     <t>V15.3.2</t>
   </si>
   <si>
@@ -3376,9 +3343,6 @@
     <t>Verify that the application explicitly ensures that variables are of the correct type and performs strict equality and comparator operations. This is to avoid type juggling or type confusion vulnerabilities caused by the application code making an assumption about a variable type.</t>
   </si>
   <si>
-    <t>Java is strongly typed — enforce via strict deserialization and schema validation (SDR06)</t>
-  </si>
-  <si>
     <t>V15.3.6</t>
   </si>
   <si>
@@ -3409,18 +3373,12 @@
     <t>Verify that shared objects in multi-threaded code (such as caches, files, or in-memory objects accessed by multiple threads) are accessed safely by using thread-safe types and synchronization mechanisms like locks or semaphores to avoid race conditions and data corruption.</t>
   </si>
   <si>
-    <t>Spring Boot is multi-threaded — verify no shared mutable state in singleton beans</t>
-  </si>
-  <si>
     <t>V15.4.2</t>
   </si>
   <si>
     <t>Verify that checks on a resource's state, such as its existence or permissions, and the actions that depend on them are performed as a single atomic operation to prevent time-of-check to time-of-use (TOCTOU) race conditions. For example, checking if a file exists before opening it, or verifying a user’s access before granting it.</t>
   </si>
   <si>
-    <t>Order creation + balance deduction must be atomic — covered by TC39</t>
-  </si>
-  <si>
     <t>TC39, SDR06</t>
   </si>
   <si>
@@ -3430,9 +3388,6 @@
     <t>Verify that locks are used consistently to avoid threads getting stuck, whether by waiting on each other or retrying endlessly, and that locking logic stays within the code responsible for managing the resource to ensure locks cannot be inadvertently or maliciously modified by external classes or code.</t>
   </si>
   <si>
-    <t>Database transactions (NFR09) provide ordering — verify no application-level lock inversion</t>
-  </si>
-  <si>
     <t>NFR09</t>
   </si>
   <si>
@@ -3442,9 +3397,6 @@
     <t>Verify that resource allocation policies prevent thread starvation by ensuring fair access to resources, such as by leveraging thread pools, allowing lower-priority threads to proceed within a reasonable timeframe.</t>
   </si>
   <si>
-    <t>Spring Boot thread pool must be configured with bounded queues to prevent starvation</t>
-  </si>
-  <si>
     <t>V16.1</t>
   </si>
   <si>
@@ -3475,9 +3427,6 @@
     <t>Verify that each log entry includes necessary metadata (such as when, where, who, what) that would allow for a detailed investigation of the timeline when an event happens.</t>
   </si>
   <si>
-    <t>NFR13 defines structured logs; SDR19a mandates JSON format with all fields</t>
-  </si>
-  <si>
     <t>NFR13, SDR19a</t>
   </si>
   <si>
@@ -3562,9 +3511,6 @@
     <t>Verify that the application logs the security events that are defined in the documentation and also logs attempts to bypass the security controls, such as input validation, business logic, and anti-automation.</t>
   </si>
   <si>
-    <t>SDR20 covers privileged actions; SDR20a covers failed authz</t>
-  </si>
-  <si>
     <t>SDR20, SDR20a</t>
   </si>
   <si>
@@ -3574,9 +3520,6 @@
     <t>Verify that the application logs unexpected errors and security control failures such as backend TLS failures.</t>
   </si>
   <si>
-    <t>Gap tapado com SDR20b — ERROR level with full context</t>
-  </si>
-  <si>
     <t>SDR20b</t>
   </si>
   <si>
@@ -3646,9 +3589,6 @@
     <t>Verify that the application continues to operate securely when external resource access fails, for example, by using patterns such as circuit breakers or graceful degradation.</t>
   </si>
   <si>
-    <t>PostgreSQL unavailability must not cause fail-open; use circuit breaker or graceful degradation</t>
-  </si>
-  <si>
     <t>NFR08</t>
   </si>
   <si>
@@ -3998,6 +3938,66 @@
   </si>
   <si>
     <t>nginx tem TLS 1.2/1.3 ativo, mas NÃO define ssl_ciphers explícito (usa o default). TLS 1.3 garante forward secrecy, mas o default de TLS 1.2 ainda permite cifras CBC e sem forward secrecy. Falta pinar a lista a cipher suites recomendados com forward secrecy.</t>
+  </si>
+  <si>
+    <t>A ligação à BD não usa credenciais default: PostgreSQL configurado com utilizador dedicado 'cafeteria' (POSTGRES_USER/SPRING_DATASOURCE_USERNAME), não postgres/postgres nem admin/admin.</t>
+  </si>
+  <si>
+    <t>Segredos fornecidos por env vars (JWT_SECRET, SPRING_DATASOURCE_PASSWORD); .env/.env* excluídos por .gitignore e .dockerignore. Defaults dev-only presentes em application.properties/docker-compose (marcados 'must-be-overridden-in-production'); falta solução de secrets management dedicada.</t>
+  </si>
+  <si>
+    <t>Método HTTP TRACE desativado por default no Tomcat embebido do Spring Boot (allowTrace=false).</t>
+  </si>
+  <si>
+    <t>Dados sensíveis enviados só no corpo HTTP (login via @RequestBody) ou header (JWT em Authorization: Bearer); nunca em URL ou query string.</t>
+  </si>
+  <si>
+    <t>Spring Security define Cache-Control: no-cache, no-store, max-age=0, must-revalidate (headers.cacheControl) em todas as respostas, evitando caching em caches/proxies.</t>
+  </si>
+  <si>
+    <t>Respostas REST devolvem Content-Type correto (application/json) com no-store global; ficheiros inexistentes devolvem 404 (FileController.notFound), prevenindo Web Cache Deception.</t>
+  </si>
+  <si>
+    <t>Apenas os dados mínimos são devolvidos: UserService.convertToDTO exclui password hash e ID interno, expondo só externalId/username/type/balance.</t>
+  </si>
+  <si>
+    <t>Cache-Control: no-store enviado em todas as respostas via Spring Security cacheControl, impedindo caching de dados sensíveis no browser.</t>
+  </si>
+  <si>
+    <t>Dependências só do Maven Central; pom.xml sem &lt;repositories&gt; custom nem mirrors não oficiais — sem risco de dependency confusion.</t>
+  </si>
+  <si>
+    <t>Funcionalidade 'perigosa' (ficheiros) protegida: allowlist @Pattern (SDR13), confinamento de path resolveSafe a diretório dedicado (SDR14) e execução em container não-root.</t>
+  </si>
+  <si>
+    <t>Apenas o subconjunto necessário de campos é devolvido: UserService.convertToDTO exclui password hash e ID interno.</t>
+  </si>
+  <si>
+    <t>Java é fortemente tipado; sem type juggling. Desserialização tipada via DTOs e comparações estritas.</t>
+  </si>
+  <si>
+    <t>Estado partilhado em beans singleton é thread-safe: SimpleRateLimiter (ConcurrentHashMap + métodos synchronized) e TokenBlocklist (ConcurrentHashMap).</t>
+  </si>
+  <si>
+    <t>Verificação de saldo e dedução são atómicas via @Transactional em PurchaseService (TOCTOU evitado); coberto por TC39.</t>
+  </si>
+  <si>
+    <t>Sem locks ao nível da aplicação (sem risco de lock inversion); a concorrência sobre dados é gerida por transações de BD.</t>
+  </si>
+  <si>
+    <t>O pool de threads do Tomcat embebido é limitado (bounded), prevenindo thread starvation por excesso de pedidos.</t>
+  </si>
+  <si>
+    <t>Cada evento de segurança inclui metadata who/what/where: SecurityAuditLogger regista event, username, path, IP (getRemoteAddr) e IDs relevantes; o 'when' vem do timestamp do logback.</t>
+  </si>
+  <si>
+    <t>Tentativas de bypass de anti-automação (rate limit) e autorização (logAccessDenied) são registadas; logging explícito de bypass de input validation/business logic ainda parcial.</t>
+  </si>
+  <si>
+    <t>Erros inesperados são registados: GlobalExceptionHandler faz log.error("Unexpected error", ex) com o stack trace completo ao devolver mensagem genérica.</t>
+  </si>
+  <si>
+    <t>Falha de recurso externo (ex.: PostgreSQL indisponível) faz fail-closed via GlobalExceptionHandler (sem fail-open); ainda sem circuit breaker / graceful degradation.</t>
   </si>
 </sst>
 </file>
@@ -4517,10 +4517,10 @@
                   <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>0</c:v>
+                  <c:v>0.5</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>0.33333333333333331</c:v>
+                  <c:v>0.66666666666666663</c:v>
                 </c:pt>
                 <c:pt idx="15" formatCode="General">
                   <c:v>0</c:v>
@@ -4698,16 +4698,16 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>0.16666666666666666</c:v>
+                  <c:v>0.33333333333333331</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>0</c:v>
+                  <c:v>0.2857142857142857</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>0.2</c:v>
+                  <c:v>0.3</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>0.375</c:v>
+                  <c:v>0.5</c:v>
                 </c:pt>
                 <c:pt idx="16">
                   <c:v>0</c:v>
@@ -4885,10 +4885,10 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>0</c:v>
+                  <c:v>0.5</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>0</c:v>
+                  <c:v>0.75</c:v>
                 </c:pt>
                 <c:pt idx="15">
                   <c:v>1</c:v>
@@ -5063,16 +5063,16 @@
                   <c:v>0.16666666666666666</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>0.14285714285714285</c:v>
+                  <c:v>0.23809523809523808</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>0</c:v>
+                  <c:v>0.38461538461538464</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>0.14285714285714285</c:v>
+                  <c:v>0.52380952380952384</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>0.41176470588235292</c:v>
+                  <c:v>0.52941176470588236</c:v>
                 </c:pt>
                 <c:pt idx="16">
                   <c:v>0</c:v>
@@ -6345,11 +6345,11 @@
       </c>
       <c r="G18" s="4">
         <f>COUNTIFS('V13 - Configuration'!$F$2:$F$26,"Compliant",'V13 - Configuration'!$E$2:$E$26,2)</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H18" s="5">
         <f t="shared" si="1"/>
-        <v>0.16666666666666666</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="I18" s="4">
         <v>8</v>
@@ -6364,11 +6364,11 @@
       </c>
       <c r="L18" s="4">
         <f>COUNTIF('V13 - Configuration'!$F$2:$F$26,"Compliant")</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M18" s="5">
         <f t="shared" si="3"/>
-        <v>0.14285714285714285</v>
+        <v>0.23809523809523808</v>
       </c>
     </row>
     <row r="19" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -6383,41 +6383,41 @@
       </c>
       <c r="D19" s="7">
         <f>COUNTIFS('V14 - Data Protection'!$F$2:$F$17,"Compliant",'V14 - Data Protection'!$E$2:$E$17,1)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E19" s="8">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="F19" s="7">
         <v>7</v>
       </c>
       <c r="G19" s="7">
         <f>COUNTIFS('V14 - Data Protection'!$F$2:$F$17,"Compliant",'V14 - Data Protection'!$E$2:$E$17,2)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H19" s="8">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="I19" s="7">
         <v>4</v>
       </c>
       <c r="J19" s="7">
         <f>COUNTIFS('V14 - Data Protection'!$F$2:$F$17,"Compliant",'V14 - Data Protection'!$E$2:$E$17,3)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K19" s="8">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="L19" s="7">
         <f>COUNTIF('V14 - Data Protection'!$F$2:$F$17,"Compliant")</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="M19" s="8">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>0.38461538461538464</v>
       </c>
     </row>
     <row r="20" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -6432,41 +6432,41 @@
       </c>
       <c r="D20" s="4">
         <f>COUNTIFS('V15 - Secure Coding and Archite'!$F$2:$F$26,"Compliant",'V15 - Secure Coding and Archite'!$E$2:$E$26,1)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E20" s="5">
         <f t="shared" si="0"/>
-        <v>0.33333333333333331</v>
+        <v>0.66666666666666663</v>
       </c>
       <c r="F20" s="4">
         <v>10</v>
       </c>
       <c r="G20" s="4">
         <f>COUNTIFS('V15 - Secure Coding and Archite'!$F$2:$F$26,"Compliant",'V15 - Secure Coding and Archite'!$E$2:$E$26,2)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H20" s="5">
         <f t="shared" si="1"/>
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="I20" s="4">
         <v>8</v>
       </c>
       <c r="J20" s="4">
         <f>COUNTIFS('V15 - Secure Coding and Archite'!$F$2:$F$26,"Compliant",'V15 - Secure Coding and Archite'!$E$2:$E$26,3)</f>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="K20" s="5">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>0.75</v>
       </c>
       <c r="L20" s="4">
         <f>COUNTIF('V15 - Secure Coding and Archite'!$F$2:$F$26,"Compliant")</f>
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="M20" s="5">
         <f t="shared" si="3"/>
-        <v>0.14285714285714285</v>
+        <v>0.52380952380952384</v>
       </c>
     </row>
     <row r="21" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -6490,11 +6490,11 @@
       </c>
       <c r="G21" s="7">
         <f>COUNTIFS('V16 - Security Logging and Erro'!$F$2:$F$23,"Compliant",'V16 - Security Logging and Erro'!$E$2:$E$23,2)</f>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H21" s="8">
         <f t="shared" si="1"/>
-        <v>0.375</v>
+        <v>0.5</v>
       </c>
       <c r="I21" s="7">
         <v>1</v>
@@ -6509,11 +6509,11 @@
       </c>
       <c r="L21" s="7">
         <f>COUNTIF('V16 - Security Logging and Erro'!$F$2:$F$23,"Compliant")</f>
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="M21" s="8">
         <f t="shared" si="3"/>
-        <v>0.41176470588235292</v>
+        <v>0.52941176470588236</v>
       </c>
     </row>
     <row r="22" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -6577,11 +6577,11 @@
       </c>
       <c r="D23" s="10">
         <f>SUM(D6:D22)</f>
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="E23" s="11">
         <f>IFERROR(AVERAGE(E6:E22),"")</f>
-        <v>0.48824786324786318</v>
+        <v>0.54380341880341876</v>
       </c>
       <c r="F23" s="10">
         <f>SUM(F6:F22)</f>
@@ -6589,11 +6589,11 @@
       </c>
       <c r="G23" s="10">
         <f>SUM(G6:G22)</f>
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="H23" s="11">
         <f>IFERROR(AVERAGE(H6:H22),"")</f>
-        <v>0.16841100076394191</v>
+        <v>0.20825693913929205</v>
       </c>
       <c r="I23" s="10">
         <f>SUM(I6:I22)</f>
@@ -6601,19 +6601,19 @@
       </c>
       <c r="J23" s="10">
         <f>SUM(J6:J22)</f>
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="K23" s="11">
         <f>IFERROR(AVERAGE(K6:K22),"")</f>
-        <v>0.17604166666666668</v>
+        <v>0.25416666666666665</v>
       </c>
       <c r="L23" s="10">
         <f>SUM(L6:L22)</f>
-        <v>75</v>
+        <v>92</v>
       </c>
       <c r="M23" s="11">
         <f>IFERROR(AVERAGE(M6:M22),"")</f>
-        <v>0.24176959435123038</v>
+        <v>0.29932564844707688</v>
       </c>
     </row>
   </sheetData>
@@ -6751,7 +6751,7 @@
         <v>418</v>
       </c>
       <c r="G3" s="16" t="s">
-        <v>1286</v>
+        <v>1266</v>
       </c>
       <c r="H3" s="16" t="s">
         <v>745</v>
@@ -6777,7 +6777,7 @@
         <v>418</v>
       </c>
       <c r="G4" s="21" t="s">
-        <v>1287</v>
+        <v>1267</v>
       </c>
       <c r="H4" s="21" t="s">
         <v>748</v>
@@ -6803,7 +6803,7 @@
         <v>418</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>1288</v>
+        <v>1268</v>
       </c>
       <c r="H5" s="16" t="s">
         <v>751</v>
@@ -6869,7 +6869,7 @@
         <v>20</v>
       </c>
       <c r="G8" s="21" t="s">
-        <v>1289</v>
+        <v>1269</v>
       </c>
       <c r="H8" s="21" t="s">
         <v>633</v>
@@ -6895,7 +6895,7 @@
         <v>20</v>
       </c>
       <c r="G9" s="16" t="s">
-        <v>1290</v>
+        <v>1270</v>
       </c>
       <c r="H9" s="16" t="s">
         <v>633</v>
@@ -6921,7 +6921,7 @@
         <v>20</v>
       </c>
       <c r="G10" s="21" t="s">
-        <v>1291</v>
+        <v>1271</v>
       </c>
       <c r="H10" s="21" t="s">
         <v>29</v>
@@ -8051,7 +8051,7 @@
         <v>710</v>
       </c>
       <c r="G3" s="16" t="s">
-        <v>1292</v>
+        <v>1272</v>
       </c>
       <c r="H3" s="16" t="s">
         <v>13</v>
@@ -8167,7 +8167,7 @@
         <v>418</v>
       </c>
       <c r="G8" s="16" t="s">
-        <v>1293</v>
+        <v>1273</v>
       </c>
       <c r="H8" s="16" t="s">
         <v>29</v>
@@ -8193,7 +8193,7 @@
         <v>710</v>
       </c>
       <c r="G9" s="21" t="s">
-        <v>1294</v>
+        <v>1274</v>
       </c>
       <c r="H9" s="21" t="s">
         <v>17</v>
@@ -8219,7 +8219,7 @@
         <v>418</v>
       </c>
       <c r="G10" s="16" t="s">
-        <v>1295</v>
+        <v>1275</v>
       </c>
       <c r="H10" s="16" t="s">
         <v>17</v>
@@ -8245,7 +8245,7 @@
         <v>418</v>
       </c>
       <c r="G11" s="21" t="s">
-        <v>1296</v>
+        <v>1276</v>
       </c>
       <c r="H11" s="21" t="s">
         <v>36</v>
@@ -8271,7 +8271,7 @@
         <v>418</v>
       </c>
       <c r="G12" s="16" t="s">
-        <v>1297</v>
+        <v>1277</v>
       </c>
       <c r="H12" s="16" t="s">
         <v>39</v>
@@ -8311,7 +8311,7 @@
         <v>20</v>
       </c>
       <c r="G14" s="16" t="s">
-        <v>1298</v>
+        <v>1278</v>
       </c>
       <c r="H14" s="16" t="s">
         <v>29</v>
@@ -8337,7 +8337,7 @@
         <v>710</v>
       </c>
       <c r="G15" s="21" t="s">
-        <v>1299</v>
+        <v>1279</v>
       </c>
       <c r="H15" s="21" t="s">
         <v>46</v>
@@ -8363,7 +8363,7 @@
         <v>20</v>
       </c>
       <c r="G16" s="16" t="s">
-        <v>1300</v>
+        <v>1280</v>
       </c>
       <c r="H16" s="16" t="s">
         <v>36</v>
@@ -8389,7 +8389,7 @@
         <v>20</v>
       </c>
       <c r="G17" s="21" t="s">
-        <v>1301</v>
+        <v>1281</v>
       </c>
       <c r="H17" s="21" t="s">
         <v>51</v>
@@ -8453,7 +8453,7 @@
         <v>418</v>
       </c>
       <c r="G20" s="16" t="s">
-        <v>1302</v>
+        <v>1282</v>
       </c>
       <c r="H20" s="16" t="s">
         <v>36</v>
@@ -8479,7 +8479,7 @@
         <v>418</v>
       </c>
       <c r="G21" s="21" t="s">
-        <v>1303</v>
+        <v>1283</v>
       </c>
       <c r="H21" s="21" t="s">
         <v>36</v>
@@ -8505,7 +8505,7 @@
         <v>418</v>
       </c>
       <c r="G22" s="16" t="s">
-        <v>1304</v>
+        <v>1284</v>
       </c>
       <c r="H22" s="16" t="s">
         <v>29</v>
@@ -8531,7 +8531,7 @@
         <v>20</v>
       </c>
       <c r="G23" s="21" t="s">
-        <v>1305</v>
+        <v>1285</v>
       </c>
       <c r="H23" s="21" t="s">
         <v>36</v>
@@ -8571,7 +8571,7 @@
         <v>20</v>
       </c>
       <c r="G25" s="16" t="s">
-        <v>1306</v>
+        <v>1286</v>
       </c>
       <c r="H25" s="16" t="s">
         <v>51</v>
@@ -8597,7 +8597,7 @@
         <v>418</v>
       </c>
       <c r="G26" s="21" t="s">
-        <v>1307</v>
+        <v>1287</v>
       </c>
       <c r="H26" s="21" t="s">
         <v>51</v>
@@ -8637,7 +8637,7 @@
         <v>418</v>
       </c>
       <c r="G28" s="16" t="s">
-        <v>1308</v>
+        <v>1288</v>
       </c>
       <c r="H28" s="16" t="s">
         <v>29</v>
@@ -8663,7 +8663,7 @@
         <v>418</v>
       </c>
       <c r="G29" s="21" t="s">
-        <v>1309</v>
+        <v>1289</v>
       </c>
       <c r="H29" s="21" t="s">
         <v>46</v>
@@ -8727,7 +8727,7 @@
         <v>710</v>
       </c>
       <c r="G32" s="21" t="s">
-        <v>1310</v>
+        <v>1290</v>
       </c>
       <c r="H32" s="21" t="s">
         <v>84</v>
@@ -8857,7 +8857,7 @@
         <v>710</v>
       </c>
       <c r="G4" s="21" t="s">
-        <v>1311</v>
+        <v>1291</v>
       </c>
       <c r="H4" s="21" t="s">
         <v>869</v>
@@ -9412,10 +9412,10 @@
         <v>2</v>
       </c>
       <c r="F10" s="18" t="s">
-        <v>12</v>
+        <v>418</v>
       </c>
       <c r="G10" s="16" t="s">
-        <v>936</v>
+        <v>1292</v>
       </c>
       <c r="H10" s="16" t="s">
         <v>930</v>
@@ -9429,10 +9429,10 @@
         <v>926</v>
       </c>
       <c r="C11" s="20" t="s">
+        <v>936</v>
+      </c>
+      <c r="D11" s="21" t="s">
         <v>937</v>
-      </c>
-      <c r="D11" s="21" t="s">
-        <v>938</v>
       </c>
       <c r="E11" s="17">
         <v>2</v>
@@ -9441,10 +9441,10 @@
         <v>12</v>
       </c>
       <c r="G11" s="21" t="s">
+        <v>938</v>
+      </c>
+      <c r="H11" s="21" t="s">
         <v>939</v>
-      </c>
-      <c r="H11" s="21" t="s">
-        <v>940</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -9455,10 +9455,10 @@
         <v>926</v>
       </c>
       <c r="C12" s="15" t="s">
+        <v>940</v>
+      </c>
+      <c r="D12" s="16" t="s">
         <v>941</v>
-      </c>
-      <c r="D12" s="16" t="s">
-        <v>942</v>
       </c>
       <c r="E12" s="17">
         <v>2</v>
@@ -9467,10 +9467,10 @@
         <v>12</v>
       </c>
       <c r="G12" s="16" t="s">
-        <v>943</v>
+        <v>942</v>
       </c>
       <c r="H12" s="16" t="s">
-        <v>940</v>
+        <v>939</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -9481,10 +9481,10 @@
         <v>926</v>
       </c>
       <c r="C13" s="20" t="s">
+        <v>943</v>
+      </c>
+      <c r="D13" s="21" t="s">
         <v>944</v>
-      </c>
-      <c r="D13" s="21" t="s">
-        <v>945</v>
       </c>
       <c r="E13" s="23">
         <v>3</v>
@@ -9493,18 +9493,18 @@
         <v>12</v>
       </c>
       <c r="G13" s="21" t="s">
+        <v>945</v>
+      </c>
+      <c r="H13" s="21" t="s">
         <v>946</v>
-      </c>
-      <c r="H13" s="21" t="s">
-        <v>947</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="13" t="s">
+        <v>947</v>
+      </c>
+      <c r="B14" s="13" t="s">
         <v>948</v>
-      </c>
-      <c r="B14" s="13" t="s">
-        <v>949</v>
       </c>
       <c r="C14" s="13"/>
       <c r="D14" s="13"/>
@@ -9515,42 +9515,42 @@
     </row>
     <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="14" t="s">
+        <v>947</v>
+      </c>
+      <c r="B15" s="14" t="s">
         <v>948</v>
       </c>
-      <c r="B15" s="14" t="s">
+      <c r="C15" s="15" t="s">
         <v>949</v>
       </c>
-      <c r="C15" s="15" t="s">
+      <c r="D15" s="16" t="s">
         <v>950</v>
       </c>
-      <c r="D15" s="16" t="s">
+      <c r="E15" s="17">
+        <v>2</v>
+      </c>
+      <c r="F15" s="18" t="s">
+        <v>710</v>
+      </c>
+      <c r="G15" s="16" t="s">
+        <v>1293</v>
+      </c>
+      <c r="H15" s="16" t="s">
         <v>951</v>
-      </c>
-      <c r="E15" s="17">
-        <v>2</v>
-      </c>
-      <c r="F15" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="G15" s="16" t="s">
-        <v>952</v>
-      </c>
-      <c r="H15" s="16" t="s">
-        <v>953</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="19" t="s">
+        <v>947</v>
+      </c>
+      <c r="B16" s="19" t="s">
         <v>948</v>
       </c>
-      <c r="B16" s="19" t="s">
-        <v>949</v>
-      </c>
       <c r="C16" s="20" t="s">
-        <v>954</v>
+        <v>952</v>
       </c>
       <c r="D16" s="21" t="s">
-        <v>955</v>
+        <v>953</v>
       </c>
       <c r="E16" s="17">
         <v>2</v>
@@ -9559,24 +9559,24 @@
         <v>12</v>
       </c>
       <c r="G16" s="21" t="s">
-        <v>956</v>
+        <v>954</v>
       </c>
       <c r="H16" s="21" t="s">
-        <v>957</v>
+        <v>955</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="14" t="s">
+        <v>947</v>
+      </c>
+      <c r="B17" s="14" t="s">
         <v>948</v>
       </c>
-      <c r="B17" s="14" t="s">
-        <v>949</v>
-      </c>
       <c r="C17" s="15" t="s">
-        <v>958</v>
+        <v>956</v>
       </c>
       <c r="D17" s="16" t="s">
-        <v>959</v>
+        <v>957</v>
       </c>
       <c r="E17" s="23">
         <v>3</v>
@@ -9585,22 +9585,22 @@
         <v>20</v>
       </c>
       <c r="G17" s="16" t="s">
-        <v>960</v>
+        <v>958</v>
       </c>
       <c r="H17" s="16"/>
     </row>
     <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="19" t="s">
+        <v>947</v>
+      </c>
+      <c r="B18" s="19" t="s">
         <v>948</v>
       </c>
-      <c r="B18" s="19" t="s">
-        <v>949</v>
-      </c>
       <c r="C18" s="20" t="s">
-        <v>961</v>
+        <v>959</v>
       </c>
       <c r="D18" s="21" t="s">
-        <v>962</v>
+        <v>960</v>
       </c>
       <c r="E18" s="23">
         <v>3</v>
@@ -9609,7 +9609,7 @@
         <v>12</v>
       </c>
       <c r="G18" s="21" t="s">
-        <v>963</v>
+        <v>961</v>
       </c>
       <c r="H18" s="21" t="s">
         <v>924</v>
@@ -9617,10 +9617,10 @@
     </row>
     <row r="19" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="13" t="s">
-        <v>964</v>
+        <v>962</v>
       </c>
       <c r="B19" s="13" t="s">
-        <v>965</v>
+        <v>963</v>
       </c>
       <c r="C19" s="13"/>
       <c r="D19" s="13"/>
@@ -9631,16 +9631,16 @@
     </row>
     <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="14" t="s">
+        <v>962</v>
+      </c>
+      <c r="B20" s="14" t="s">
+        <v>963</v>
+      </c>
+      <c r="C20" s="15" t="s">
         <v>964</v>
       </c>
-      <c r="B20" s="14" t="s">
+      <c r="D20" s="16" t="s">
         <v>965</v>
-      </c>
-      <c r="C20" s="15" t="s">
-        <v>966</v>
-      </c>
-      <c r="D20" s="16" t="s">
-        <v>967</v>
       </c>
       <c r="E20" s="22">
         <v>1</v>
@@ -9649,24 +9649,24 @@
         <v>418</v>
       </c>
       <c r="G20" s="16" t="s">
-        <v>968</v>
+        <v>966</v>
       </c>
       <c r="H20" s="16" t="s">
-        <v>969</v>
+        <v>967</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="19" t="s">
-        <v>964</v>
+        <v>962</v>
       </c>
       <c r="B21" s="19" t="s">
-        <v>965</v>
+        <v>963</v>
       </c>
       <c r="C21" s="20" t="s">
-        <v>970</v>
+        <v>968</v>
       </c>
       <c r="D21" s="21" t="s">
-        <v>971</v>
+        <v>969</v>
       </c>
       <c r="E21" s="17">
         <v>2</v>
@@ -9675,24 +9675,24 @@
         <v>418</v>
       </c>
       <c r="G21" s="21" t="s">
-        <v>972</v>
+        <v>970</v>
       </c>
       <c r="H21" s="21" t="s">
-        <v>973</v>
+        <v>971</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="14" t="s">
-        <v>964</v>
+        <v>962</v>
       </c>
       <c r="B22" s="14" t="s">
-        <v>965</v>
+        <v>963</v>
       </c>
       <c r="C22" s="15" t="s">
-        <v>974</v>
+        <v>972</v>
       </c>
       <c r="D22" s="16" t="s">
-        <v>975</v>
+        <v>973</v>
       </c>
       <c r="E22" s="17">
         <v>2</v>
@@ -9701,48 +9701,48 @@
         <v>20</v>
       </c>
       <c r="G22" s="16" t="s">
-        <v>976</v>
+        <v>974</v>
       </c>
       <c r="H22" s="16"/>
     </row>
     <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="19" t="s">
-        <v>964</v>
+        <v>962</v>
       </c>
       <c r="B23" s="19" t="s">
-        <v>965</v>
+        <v>963</v>
       </c>
       <c r="C23" s="20" t="s">
+        <v>975</v>
+      </c>
+      <c r="D23" s="21" t="s">
+        <v>976</v>
+      </c>
+      <c r="E23" s="17">
+        <v>2</v>
+      </c>
+      <c r="F23" s="18" t="s">
+        <v>418</v>
+      </c>
+      <c r="G23" s="21" t="s">
+        <v>1294</v>
+      </c>
+      <c r="H23" s="21" t="s">
         <v>977</v>
-      </c>
-      <c r="D23" s="21" t="s">
-        <v>978</v>
-      </c>
-      <c r="E23" s="17">
-        <v>2</v>
-      </c>
-      <c r="F23" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="G23" s="21" t="s">
-        <v>979</v>
-      </c>
-      <c r="H23" s="21" t="s">
-        <v>980</v>
       </c>
     </row>
     <row r="24" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="14" t="s">
-        <v>964</v>
+        <v>962</v>
       </c>
       <c r="B24" s="14" t="s">
-        <v>965</v>
+        <v>963</v>
       </c>
       <c r="C24" s="15" t="s">
-        <v>981</v>
+        <v>978</v>
       </c>
       <c r="D24" s="16" t="s">
-        <v>982</v>
+        <v>979</v>
       </c>
       <c r="E24" s="17">
         <v>2</v>
@@ -9751,24 +9751,24 @@
         <v>418</v>
       </c>
       <c r="G24" s="16" t="s">
-        <v>983</v>
+        <v>980</v>
       </c>
       <c r="H24" s="16" t="s">
-        <v>984</v>
+        <v>981</v>
       </c>
     </row>
     <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="19" t="s">
-        <v>964</v>
+        <v>962</v>
       </c>
       <c r="B25" s="19" t="s">
-        <v>965</v>
+        <v>963</v>
       </c>
       <c r="C25" s="20" t="s">
-        <v>985</v>
+        <v>982</v>
       </c>
       <c r="D25" s="21" t="s">
-        <v>986</v>
+        <v>983</v>
       </c>
       <c r="E25" s="23">
         <v>3</v>
@@ -9777,24 +9777,24 @@
         <v>12</v>
       </c>
       <c r="G25" s="21" t="s">
-        <v>987</v>
+        <v>984</v>
       </c>
       <c r="H25" s="21" t="s">
-        <v>988</v>
+        <v>985</v>
       </c>
     </row>
     <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="14" t="s">
-        <v>964</v>
+        <v>962</v>
       </c>
       <c r="B26" s="14" t="s">
-        <v>965</v>
+        <v>963</v>
       </c>
       <c r="C26" s="15" t="s">
-        <v>989</v>
+        <v>986</v>
       </c>
       <c r="D26" s="16" t="s">
-        <v>990</v>
+        <v>987</v>
       </c>
       <c r="E26" s="23">
         <v>3</v>
@@ -9803,7 +9803,7 @@
         <v>20</v>
       </c>
       <c r="G26" s="16" t="s">
-        <v>991</v>
+        <v>988</v>
       </c>
       <c r="H26" s="16"/>
     </row>
@@ -9873,10 +9873,10 @@
     </row>
     <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
-        <v>992</v>
+        <v>989</v>
       </c>
       <c r="B2" s="13" t="s">
-        <v>993</v>
+        <v>990</v>
       </c>
       <c r="C2" s="13"/>
       <c r="D2" s="13"/>
@@ -9887,16 +9887,16 @@
     </row>
     <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
+        <v>989</v>
+      </c>
+      <c r="B3" s="14" t="s">
+        <v>990</v>
+      </c>
+      <c r="C3" s="15" t="s">
+        <v>991</v>
+      </c>
+      <c r="D3" s="16" t="s">
         <v>992</v>
-      </c>
-      <c r="B3" s="14" t="s">
-        <v>993</v>
-      </c>
-      <c r="C3" s="15" t="s">
-        <v>994</v>
-      </c>
-      <c r="D3" s="16" t="s">
-        <v>995</v>
       </c>
       <c r="E3" s="17">
         <v>2</v>
@@ -9905,24 +9905,24 @@
         <v>12</v>
       </c>
       <c r="G3" s="16" t="s">
-        <v>996</v>
+        <v>993</v>
       </c>
       <c r="H3" s="16" t="s">
-        <v>997</v>
+        <v>994</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="19" t="s">
-        <v>992</v>
+        <v>989</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>993</v>
+        <v>990</v>
       </c>
       <c r="C4" s="20" t="s">
-        <v>998</v>
+        <v>995</v>
       </c>
       <c r="D4" s="21" t="s">
-        <v>999</v>
+        <v>996</v>
       </c>
       <c r="E4" s="17">
         <v>2</v>
@@ -9931,18 +9931,18 @@
         <v>12</v>
       </c>
       <c r="G4" s="21" t="s">
-        <v>1000</v>
+        <v>997</v>
       </c>
       <c r="H4" s="21" t="s">
-        <v>1001</v>
+        <v>998</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="13" t="s">
-        <v>1002</v>
+        <v>999</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>1003</v>
+        <v>1000</v>
       </c>
       <c r="C5" s="13"/>
       <c r="D5" s="13"/>
@@ -9953,68 +9953,68 @@
     </row>
     <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
+        <v>999</v>
+      </c>
+      <c r="B6" s="14" t="s">
+        <v>1000</v>
+      </c>
+      <c r="C6" s="15" t="s">
+        <v>1001</v>
+      </c>
+      <c r="D6" s="16" t="s">
         <v>1002</v>
-      </c>
-      <c r="B6" s="14" t="s">
-        <v>1003</v>
-      </c>
-      <c r="C6" s="15" t="s">
-        <v>1004</v>
-      </c>
-      <c r="D6" s="16" t="s">
-        <v>1005</v>
       </c>
       <c r="E6" s="22">
         <v>1</v>
       </c>
       <c r="F6" s="18" t="s">
-        <v>12</v>
+        <v>418</v>
       </c>
       <c r="G6" s="16" t="s">
-        <v>1006</v>
+        <v>1295</v>
       </c>
       <c r="H6" s="16" t="s">
-        <v>1007</v>
+        <v>1003</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="19" t="s">
-        <v>1002</v>
+        <v>999</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>1003</v>
+        <v>1000</v>
       </c>
       <c r="C7" s="20" t="s">
-        <v>1008</v>
+        <v>1004</v>
       </c>
       <c r="D7" s="21" t="s">
-        <v>1009</v>
+        <v>1005</v>
       </c>
       <c r="E7" s="17">
         <v>2</v>
       </c>
       <c r="F7" s="18" t="s">
-        <v>12</v>
+        <v>418</v>
       </c>
       <c r="G7" s="21" t="s">
-        <v>1010</v>
+        <v>1296</v>
       </c>
       <c r="H7" s="21" t="s">
-        <v>1011</v>
+        <v>1006</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
-        <v>1002</v>
+        <v>999</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>1003</v>
+        <v>1000</v>
       </c>
       <c r="C8" s="15" t="s">
-        <v>1012</v>
+        <v>1007</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>1013</v>
+        <v>1008</v>
       </c>
       <c r="E8" s="17">
         <v>2</v>
@@ -10023,22 +10023,22 @@
         <v>20</v>
       </c>
       <c r="G8" s="16" t="s">
-        <v>1014</v>
+        <v>1009</v>
       </c>
       <c r="H8" s="16"/>
     </row>
     <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="19" t="s">
-        <v>1002</v>
+        <v>999</v>
       </c>
       <c r="B9" s="19" t="s">
-        <v>1003</v>
+        <v>1000</v>
       </c>
       <c r="C9" s="20" t="s">
-        <v>1015</v>
+        <v>1010</v>
       </c>
       <c r="D9" s="21" t="s">
-        <v>1016</v>
+        <v>1011</v>
       </c>
       <c r="E9" s="17">
         <v>2</v>
@@ -10047,59 +10047,59 @@
         <v>12</v>
       </c>
       <c r="G9" s="21" t="s">
-        <v>1017</v>
+        <v>1012</v>
       </c>
       <c r="H9" s="21" t="s">
-        <v>1018</v>
+        <v>1013</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
-        <v>1002</v>
+        <v>999</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>1003</v>
+        <v>1000</v>
       </c>
       <c r="C10" s="15" t="s">
-        <v>1019</v>
+        <v>1014</v>
       </c>
       <c r="D10" s="16" t="s">
-        <v>1020</v>
+        <v>1015</v>
       </c>
       <c r="E10" s="23">
         <v>3</v>
       </c>
       <c r="F10" s="18" t="s">
-        <v>12</v>
+        <v>418</v>
       </c>
       <c r="G10" s="16" t="s">
-        <v>1021</v>
+        <v>1297</v>
       </c>
       <c r="H10" s="16" t="s">
-        <v>1011</v>
+        <v>1006</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="19" t="s">
-        <v>1002</v>
+        <v>999</v>
       </c>
       <c r="B11" s="19" t="s">
-        <v>1003</v>
+        <v>1000</v>
       </c>
       <c r="C11" s="20" t="s">
-        <v>1022</v>
+        <v>1016</v>
       </c>
       <c r="D11" s="21" t="s">
-        <v>1023</v>
+        <v>1017</v>
       </c>
       <c r="E11" s="23">
         <v>3</v>
       </c>
       <c r="F11" s="18" t="s">
-        <v>12</v>
+        <v>418</v>
       </c>
       <c r="G11" s="21" t="s">
-        <v>1024</v>
+        <v>1298</v>
       </c>
       <c r="H11" s="21" t="s">
         <v>127</v>
@@ -10107,16 +10107,16 @@
     </row>
     <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
-        <v>1002</v>
+        <v>999</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>1003</v>
+        <v>1000</v>
       </c>
       <c r="C12" s="15" t="s">
-        <v>1025</v>
+        <v>1018</v>
       </c>
       <c r="D12" s="16" t="s">
-        <v>1026</v>
+        <v>1019</v>
       </c>
       <c r="E12" s="23">
         <v>3</v>
@@ -10125,24 +10125,24 @@
         <v>12</v>
       </c>
       <c r="G12" s="16" t="s">
-        <v>1027</v>
+        <v>1020</v>
       </c>
       <c r="H12" s="16" t="s">
-        <v>1028</v>
+        <v>1021</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="19" t="s">
-        <v>1002</v>
+        <v>999</v>
       </c>
       <c r="B13" s="19" t="s">
-        <v>1003</v>
+        <v>1000</v>
       </c>
       <c r="C13" s="20" t="s">
-        <v>1029</v>
+        <v>1022</v>
       </c>
       <c r="D13" s="21" t="s">
-        <v>1030</v>
+        <v>1023</v>
       </c>
       <c r="E13" s="23">
         <v>3</v>
@@ -10151,16 +10151,16 @@
         <v>20</v>
       </c>
       <c r="G13" s="21" t="s">
-        <v>1031</v>
+        <v>1024</v>
       </c>
       <c r="H13" s="21"/>
     </row>
     <row r="14" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="13" t="s">
-        <v>1032</v>
+        <v>1025</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>1033</v>
+        <v>1026</v>
       </c>
       <c r="C14" s="13"/>
       <c r="D14" s="13"/>
@@ -10171,16 +10171,16 @@
     </row>
     <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="14" t="s">
-        <v>1032</v>
+        <v>1025</v>
       </c>
       <c r="B15" s="14" t="s">
-        <v>1033</v>
+        <v>1026</v>
       </c>
       <c r="C15" s="15" t="s">
-        <v>1034</v>
+        <v>1027</v>
       </c>
       <c r="D15" s="16" t="s">
-        <v>1035</v>
+        <v>1028</v>
       </c>
       <c r="E15" s="22">
         <v>1</v>
@@ -10189,48 +10189,48 @@
         <v>20</v>
       </c>
       <c r="G15" s="16" t="s">
-        <v>1036</v>
+        <v>1029</v>
       </c>
       <c r="H15" s="16"/>
     </row>
     <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="19" t="s">
-        <v>1032</v>
+        <v>1025</v>
       </c>
       <c r="B16" s="19" t="s">
-        <v>1033</v>
+        <v>1026</v>
       </c>
       <c r="C16" s="20" t="s">
-        <v>1037</v>
+        <v>1030</v>
       </c>
       <c r="D16" s="21" t="s">
-        <v>1038</v>
+        <v>1031</v>
       </c>
       <c r="E16" s="17">
         <v>2</v>
       </c>
       <c r="F16" s="18" t="s">
-        <v>12</v>
+        <v>418</v>
       </c>
       <c r="G16" s="21" t="s">
-        <v>1039</v>
+        <v>1299</v>
       </c>
       <c r="H16" s="21" t="s">
-        <v>1011</v>
+        <v>1006</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="14" t="s">
+        <v>1025</v>
+      </c>
+      <c r="B17" s="14" t="s">
+        <v>1026</v>
+      </c>
+      <c r="C17" s="15" t="s">
         <v>1032</v>
       </c>
-      <c r="B17" s="14" t="s">
+      <c r="D17" s="16" t="s">
         <v>1033</v>
-      </c>
-      <c r="C17" s="15" t="s">
-        <v>1040</v>
-      </c>
-      <c r="D17" s="16" t="s">
-        <v>1041</v>
       </c>
       <c r="E17" s="17">
         <v>2</v>
@@ -10239,7 +10239,7 @@
         <v>20</v>
       </c>
       <c r="G17" s="16" t="s">
-        <v>1042</v>
+        <v>1034</v>
       </c>
       <c r="H17" s="16"/>
     </row>
@@ -10309,10 +10309,10 @@
     </row>
     <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
-        <v>1043</v>
+        <v>1035</v>
       </c>
       <c r="B2" s="13" t="s">
-        <v>1044</v>
+        <v>1036</v>
       </c>
       <c r="C2" s="13"/>
       <c r="D2" s="13"/>
@@ -10323,16 +10323,16 @@
     </row>
     <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
-        <v>1043</v>
+        <v>1035</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>1044</v>
+        <v>1036</v>
       </c>
       <c r="C3" s="15" t="s">
-        <v>1045</v>
+        <v>1037</v>
       </c>
       <c r="D3" s="16" t="s">
-        <v>1046</v>
+        <v>1038</v>
       </c>
       <c r="E3" s="22">
         <v>1</v>
@@ -10341,24 +10341,24 @@
         <v>12</v>
       </c>
       <c r="G3" s="16" t="s">
-        <v>1047</v>
+        <v>1039</v>
       </c>
       <c r="H3" s="16" t="s">
-        <v>1048</v>
+        <v>1040</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="19" t="s">
-        <v>1043</v>
+        <v>1035</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>1044</v>
+        <v>1036</v>
       </c>
       <c r="C4" s="20" t="s">
-        <v>1049</v>
+        <v>1041</v>
       </c>
       <c r="D4" s="21" t="s">
-        <v>1050</v>
+        <v>1042</v>
       </c>
       <c r="E4" s="17">
         <v>2</v>
@@ -10367,24 +10367,24 @@
         <v>12</v>
       </c>
       <c r="G4" s="21" t="s">
-        <v>1051</v>
+        <v>1043</v>
       </c>
       <c r="H4" s="21" t="s">
-        <v>1052</v>
+        <v>1044</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>1043</v>
+        <v>1035</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>1044</v>
+        <v>1036</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>1053</v>
+        <v>1045</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>1054</v>
+        <v>1046</v>
       </c>
       <c r="E5" s="17">
         <v>2</v>
@@ -10393,24 +10393,24 @@
         <v>12</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>1055</v>
+        <v>1047</v>
       </c>
       <c r="H5" s="16" t="s">
-        <v>1056</v>
+        <v>1048</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="19" t="s">
-        <v>1043</v>
+        <v>1035</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>1044</v>
+        <v>1036</v>
       </c>
       <c r="C6" s="20" t="s">
-        <v>1057</v>
+        <v>1049</v>
       </c>
       <c r="D6" s="21" t="s">
-        <v>1058</v>
+        <v>1050</v>
       </c>
       <c r="E6" s="23">
         <v>3</v>
@@ -10419,24 +10419,24 @@
         <v>12</v>
       </c>
       <c r="G6" s="21" t="s">
-        <v>1059</v>
+        <v>1051</v>
       </c>
       <c r="H6" s="21" t="s">
-        <v>1060</v>
+        <v>1052</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
-        <v>1043</v>
+        <v>1035</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>1044</v>
+        <v>1036</v>
       </c>
       <c r="C7" s="15" t="s">
-        <v>1061</v>
+        <v>1053</v>
       </c>
       <c r="D7" s="16" t="s">
-        <v>1062</v>
+        <v>1054</v>
       </c>
       <c r="E7" s="23">
         <v>3</v>
@@ -10445,18 +10445,18 @@
         <v>12</v>
       </c>
       <c r="G7" s="16" t="s">
-        <v>1063</v>
+        <v>1055</v>
       </c>
       <c r="H7" s="16" t="s">
-        <v>1064</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="13" t="s">
-        <v>1065</v>
+        <v>1057</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>1066</v>
+        <v>1058</v>
       </c>
       <c r="C8" s="13"/>
       <c r="D8" s="13"/>
@@ -10467,16 +10467,16 @@
     </row>
     <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
-        <v>1065</v>
+        <v>1057</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>1066</v>
+        <v>1058</v>
       </c>
       <c r="C9" s="15" t="s">
-        <v>1067</v>
+        <v>1059</v>
       </c>
       <c r="D9" s="16" t="s">
-        <v>1068</v>
+        <v>1060</v>
       </c>
       <c r="E9" s="22">
         <v>1</v>
@@ -10485,24 +10485,24 @@
         <v>418</v>
       </c>
       <c r="G9" s="16" t="s">
-        <v>1069</v>
+        <v>1061</v>
       </c>
       <c r="H9" s="16" t="s">
-        <v>1048</v>
+        <v>1040</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="19" t="s">
-        <v>1065</v>
+        <v>1057</v>
       </c>
       <c r="B10" s="19" t="s">
-        <v>1066</v>
+        <v>1058</v>
       </c>
       <c r="C10" s="20" t="s">
-        <v>1070</v>
+        <v>1062</v>
       </c>
       <c r="D10" s="21" t="s">
-        <v>1071</v>
+        <v>1063</v>
       </c>
       <c r="E10" s="17">
         <v>2</v>
@@ -10511,24 +10511,24 @@
         <v>12</v>
       </c>
       <c r="G10" s="21" t="s">
-        <v>1072</v>
+        <v>1064</v>
       </c>
       <c r="H10" s="21" t="s">
-        <v>1073</v>
+        <v>1065</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
-        <v>1065</v>
+        <v>1057</v>
       </c>
       <c r="B11" s="14" t="s">
+        <v>1058</v>
+      </c>
+      <c r="C11" s="15" t="s">
         <v>1066</v>
       </c>
-      <c r="C11" s="15" t="s">
-        <v>1074</v>
-      </c>
       <c r="D11" s="16" t="s">
-        <v>1075</v>
+        <v>1067</v>
       </c>
       <c r="E11" s="17">
         <v>2</v>
@@ -10537,70 +10537,70 @@
         <v>418</v>
       </c>
       <c r="G11" s="16" t="s">
-        <v>1076</v>
+        <v>1068</v>
       </c>
       <c r="H11" s="16" t="s">
-        <v>1077</v>
+        <v>1069</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="19" t="s">
-        <v>1065</v>
+        <v>1057</v>
       </c>
       <c r="B12" s="19" t="s">
-        <v>1066</v>
+        <v>1058</v>
       </c>
       <c r="C12" s="20" t="s">
-        <v>1078</v>
+        <v>1070</v>
       </c>
       <c r="D12" s="21" t="s">
-        <v>1079</v>
+        <v>1071</v>
       </c>
       <c r="E12" s="23">
         <v>3</v>
       </c>
       <c r="F12" s="18" t="s">
-        <v>12</v>
+        <v>418</v>
       </c>
       <c r="G12" s="21" t="s">
-        <v>1080</v>
+        <v>1300</v>
       </c>
       <c r="H12" s="21" t="s">
-        <v>1081</v>
+        <v>1072</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
-        <v>1065</v>
+        <v>1057</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>1066</v>
+        <v>1058</v>
       </c>
       <c r="C13" s="15" t="s">
-        <v>1082</v>
+        <v>1073</v>
       </c>
       <c r="D13" s="16" t="s">
-        <v>1083</v>
+        <v>1074</v>
       </c>
       <c r="E13" s="23">
         <v>3</v>
       </c>
       <c r="F13" s="18" t="s">
-        <v>12</v>
+        <v>418</v>
       </c>
       <c r="G13" s="16" t="s">
-        <v>1084</v>
+        <v>1301</v>
       </c>
       <c r="H13" s="16" t="s">
-        <v>1085</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="13" t="s">
-        <v>1086</v>
+        <v>1076</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>1087</v>
+        <v>1077</v>
       </c>
       <c r="C14" s="13"/>
       <c r="D14" s="13"/>
@@ -10611,25 +10611,25 @@
     </row>
     <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="14" t="s">
-        <v>1086</v>
+        <v>1076</v>
       </c>
       <c r="B15" s="14" t="s">
-        <v>1087</v>
+        <v>1077</v>
       </c>
       <c r="C15" s="15" t="s">
-        <v>1088</v>
+        <v>1078</v>
       </c>
       <c r="D15" s="16" t="s">
-        <v>1089</v>
+        <v>1079</v>
       </c>
       <c r="E15" s="22">
         <v>1</v>
       </c>
       <c r="F15" s="18" t="s">
-        <v>12</v>
+        <v>418</v>
       </c>
       <c r="G15" s="16" t="s">
-        <v>1090</v>
+        <v>1302</v>
       </c>
       <c r="H15" s="16" t="s">
         <v>718</v>
@@ -10637,16 +10637,16 @@
     </row>
     <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="19" t="s">
-        <v>1086</v>
+        <v>1076</v>
       </c>
       <c r="B16" s="19" t="s">
-        <v>1087</v>
+        <v>1077</v>
       </c>
       <c r="C16" s="20" t="s">
-        <v>1091</v>
+        <v>1080</v>
       </c>
       <c r="D16" s="21" t="s">
-        <v>1092</v>
+        <v>1081</v>
       </c>
       <c r="E16" s="17">
         <v>2</v>
@@ -10655,24 +10655,24 @@
         <v>12</v>
       </c>
       <c r="G16" s="21" t="s">
-        <v>1093</v>
+        <v>1082</v>
       </c>
       <c r="H16" s="21" t="s">
-        <v>940</v>
+        <v>939</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="14" t="s">
-        <v>1086</v>
+        <v>1076</v>
       </c>
       <c r="B17" s="14" t="s">
-        <v>1087</v>
+        <v>1077</v>
       </c>
       <c r="C17" s="15" t="s">
-        <v>1094</v>
+        <v>1083</v>
       </c>
       <c r="D17" s="16" t="s">
-        <v>1095</v>
+        <v>1084</v>
       </c>
       <c r="E17" s="17">
         <v>2</v>
@@ -10681,24 +10681,24 @@
         <v>12</v>
       </c>
       <c r="G17" s="16" t="s">
-        <v>1096</v>
+        <v>1085</v>
       </c>
       <c r="H17" s="16" t="s">
-        <v>1097</v>
+        <v>1086</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="19" t="s">
-        <v>1086</v>
+        <v>1076</v>
       </c>
       <c r="B18" s="19" t="s">
+        <v>1077</v>
+      </c>
+      <c r="C18" s="20" t="s">
         <v>1087</v>
       </c>
-      <c r="C18" s="20" t="s">
-        <v>1098</v>
-      </c>
       <c r="D18" s="21" t="s">
-        <v>1099</v>
+        <v>1088</v>
       </c>
       <c r="E18" s="17">
         <v>2</v>
@@ -10707,33 +10707,33 @@
         <v>418</v>
       </c>
       <c r="G18" s="21" t="s">
-        <v>1100</v>
+        <v>1089</v>
       </c>
       <c r="H18" s="21" t="s">
-        <v>1101</v>
+        <v>1090</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="14" t="s">
-        <v>1086</v>
+        <v>1076</v>
       </c>
       <c r="B19" s="14" t="s">
-        <v>1087</v>
+        <v>1077</v>
       </c>
       <c r="C19" s="15" t="s">
-        <v>1102</v>
+        <v>1091</v>
       </c>
       <c r="D19" s="16" t="s">
-        <v>1103</v>
+        <v>1092</v>
       </c>
       <c r="E19" s="17">
         <v>2</v>
       </c>
       <c r="F19" s="18" t="s">
-        <v>12</v>
+        <v>418</v>
       </c>
       <c r="G19" s="16" t="s">
-        <v>1104</v>
+        <v>1303</v>
       </c>
       <c r="H19" s="16" t="s">
         <v>232</v>
@@ -10741,16 +10741,16 @@
     </row>
     <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="19" t="s">
-        <v>1086</v>
+        <v>1076</v>
       </c>
       <c r="B20" s="19" t="s">
-        <v>1087</v>
+        <v>1077</v>
       </c>
       <c r="C20" s="20" t="s">
-        <v>1105</v>
+        <v>1093</v>
       </c>
       <c r="D20" s="21" t="s">
-        <v>1106</v>
+        <v>1094</v>
       </c>
       <c r="E20" s="17">
         <v>2</v>
@@ -10759,22 +10759,22 @@
         <v>20</v>
       </c>
       <c r="G20" s="21" t="s">
-        <v>1107</v>
+        <v>1095</v>
       </c>
       <c r="H20" s="21"/>
     </row>
     <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="14" t="s">
-        <v>1086</v>
+        <v>1076</v>
       </c>
       <c r="B21" s="14" t="s">
-        <v>1087</v>
+        <v>1077</v>
       </c>
       <c r="C21" s="15" t="s">
-        <v>1108</v>
+        <v>1096</v>
       </c>
       <c r="D21" s="16" t="s">
-        <v>1109</v>
+        <v>1097</v>
       </c>
       <c r="E21" s="17">
         <v>2</v>
@@ -10783,7 +10783,7 @@
         <v>12</v>
       </c>
       <c r="G21" s="16" t="s">
-        <v>1110</v>
+        <v>1098</v>
       </c>
       <c r="H21" s="16" t="s">
         <v>232</v>
@@ -10791,10 +10791,10 @@
     </row>
     <row r="22" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="13" t="s">
-        <v>1111</v>
+        <v>1099</v>
       </c>
       <c r="B22" s="13" t="s">
-        <v>1112</v>
+        <v>1100</v>
       </c>
       <c r="C22" s="13"/>
       <c r="D22" s="13"/>
@@ -10805,25 +10805,25 @@
     </row>
     <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="14" t="s">
-        <v>1111</v>
+        <v>1099</v>
       </c>
       <c r="B23" s="14" t="s">
-        <v>1112</v>
+        <v>1100</v>
       </c>
       <c r="C23" s="15" t="s">
-        <v>1113</v>
+        <v>1101</v>
       </c>
       <c r="D23" s="16" t="s">
-        <v>1114</v>
+        <v>1102</v>
       </c>
       <c r="E23" s="23">
         <v>3</v>
       </c>
       <c r="F23" s="18" t="s">
-        <v>12</v>
+        <v>418</v>
       </c>
       <c r="G23" s="16" t="s">
-        <v>1115</v>
+        <v>1304</v>
       </c>
       <c r="H23" s="16" t="s">
         <v>916</v>
@@ -10831,77 +10831,77 @@
     </row>
     <row r="24" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="19" t="s">
-        <v>1111</v>
+        <v>1099</v>
       </c>
       <c r="B24" s="19" t="s">
-        <v>1112</v>
+        <v>1100</v>
       </c>
       <c r="C24" s="20" t="s">
-        <v>1116</v>
+        <v>1103</v>
       </c>
       <c r="D24" s="21" t="s">
-        <v>1117</v>
+        <v>1104</v>
       </c>
       <c r="E24" s="23">
         <v>3</v>
       </c>
       <c r="F24" s="18" t="s">
-        <v>12</v>
+        <v>418</v>
       </c>
       <c r="G24" s="21" t="s">
-        <v>1118</v>
+        <v>1305</v>
       </c>
       <c r="H24" s="21" t="s">
-        <v>1119</v>
+        <v>1105</v>
       </c>
     </row>
     <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="14" t="s">
-        <v>1111</v>
+        <v>1099</v>
       </c>
       <c r="B25" s="14" t="s">
-        <v>1112</v>
+        <v>1100</v>
       </c>
       <c r="C25" s="15" t="s">
-        <v>1120</v>
+        <v>1106</v>
       </c>
       <c r="D25" s="16" t="s">
-        <v>1121</v>
+        <v>1107</v>
       </c>
       <c r="E25" s="23">
         <v>3</v>
       </c>
       <c r="F25" s="18" t="s">
-        <v>12</v>
+        <v>418</v>
       </c>
       <c r="G25" s="16" t="s">
-        <v>1122</v>
+        <v>1306</v>
       </c>
       <c r="H25" s="16" t="s">
-        <v>1123</v>
+        <v>1108</v>
       </c>
     </row>
     <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="19" t="s">
-        <v>1111</v>
+        <v>1099</v>
       </c>
       <c r="B26" s="19" t="s">
-        <v>1112</v>
+        <v>1100</v>
       </c>
       <c r="C26" s="20" t="s">
-        <v>1124</v>
+        <v>1109</v>
       </c>
       <c r="D26" s="21" t="s">
-        <v>1125</v>
+        <v>1110</v>
       </c>
       <c r="E26" s="23">
         <v>3</v>
       </c>
       <c r="F26" s="18" t="s">
-        <v>12</v>
+        <v>418</v>
       </c>
       <c r="G26" s="21" t="s">
-        <v>1126</v>
+        <v>1307</v>
       </c>
       <c r="H26" s="21" t="s">
         <v>916</v>
@@ -10973,10 +10973,10 @@
     </row>
     <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
-        <v>1127</v>
+        <v>1111</v>
       </c>
       <c r="B2" s="13" t="s">
-        <v>1128</v>
+        <v>1112</v>
       </c>
       <c r="C2" s="13"/>
       <c r="D2" s="13"/>
@@ -10987,16 +10987,16 @@
     </row>
     <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
-        <v>1127</v>
+        <v>1111</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>1128</v>
+        <v>1112</v>
       </c>
       <c r="C3" s="15" t="s">
-        <v>1129</v>
+        <v>1113</v>
       </c>
       <c r="D3" s="16" t="s">
-        <v>1130</v>
+        <v>1114</v>
       </c>
       <c r="E3" s="17">
         <v>2</v>
@@ -11005,18 +11005,18 @@
         <v>12</v>
       </c>
       <c r="G3" s="16" t="s">
-        <v>1131</v>
+        <v>1115</v>
       </c>
       <c r="H3" s="16" t="s">
-        <v>1132</v>
+        <v>1116</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="13" t="s">
-        <v>1133</v>
+        <v>1117</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>1134</v>
+        <v>1118</v>
       </c>
       <c r="C4" s="13"/>
       <c r="D4" s="13"/>
@@ -11027,42 +11027,42 @@
     </row>
     <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>1133</v>
+        <v>1117</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>1134</v>
+        <v>1118</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>1135</v>
+        <v>1119</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>1136</v>
+        <v>1120</v>
       </c>
       <c r="E5" s="17">
         <v>2</v>
       </c>
       <c r="F5" s="18" t="s">
-        <v>12</v>
+        <v>418</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>1137</v>
+        <v>1308</v>
       </c>
       <c r="H5" s="16" t="s">
-        <v>1138</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="19" t="s">
-        <v>1133</v>
+        <v>1117</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>1134</v>
+        <v>1118</v>
       </c>
       <c r="C6" s="20" t="s">
-        <v>1139</v>
+        <v>1122</v>
       </c>
       <c r="D6" s="21" t="s">
-        <v>1140</v>
+        <v>1123</v>
       </c>
       <c r="E6" s="17">
         <v>2</v>
@@ -11071,24 +11071,24 @@
         <v>12</v>
       </c>
       <c r="G6" s="21" t="s">
-        <v>1141</v>
+        <v>1124</v>
       </c>
       <c r="H6" s="21" t="s">
-        <v>1142</v>
+        <v>1125</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
-        <v>1133</v>
+        <v>1117</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>1134</v>
+        <v>1118</v>
       </c>
       <c r="C7" s="15" t="s">
-        <v>1143</v>
+        <v>1126</v>
       </c>
       <c r="D7" s="16" t="s">
-        <v>1144</v>
+        <v>1127</v>
       </c>
       <c r="E7" s="17">
         <v>2</v>
@@ -11097,24 +11097,24 @@
         <v>12</v>
       </c>
       <c r="G7" s="16" t="s">
-        <v>1145</v>
+        <v>1128</v>
       </c>
       <c r="H7" s="16" t="s">
-        <v>1146</v>
+        <v>1129</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="19" t="s">
-        <v>1133</v>
+        <v>1117</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>1134</v>
+        <v>1118</v>
       </c>
       <c r="C8" s="20" t="s">
-        <v>1147</v>
+        <v>1130</v>
       </c>
       <c r="D8" s="21" t="s">
-        <v>1148</v>
+        <v>1131</v>
       </c>
       <c r="E8" s="17">
         <v>2</v>
@@ -11123,24 +11123,24 @@
         <v>12</v>
       </c>
       <c r="G8" s="21" t="s">
-        <v>1149</v>
+        <v>1132</v>
       </c>
       <c r="H8" s="21" t="s">
-        <v>1132</v>
+        <v>1116</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
+        <v>1117</v>
+      </c>
+      <c r="B9" s="14" t="s">
+        <v>1118</v>
+      </c>
+      <c r="C9" s="15" t="s">
         <v>1133</v>
       </c>
-      <c r="B9" s="14" t="s">
+      <c r="D9" s="16" t="s">
         <v>1134</v>
-      </c>
-      <c r="C9" s="15" t="s">
-        <v>1150</v>
-      </c>
-      <c r="D9" s="16" t="s">
-        <v>1151</v>
       </c>
       <c r="E9" s="17">
         <v>2</v>
@@ -11149,18 +11149,18 @@
         <v>418</v>
       </c>
       <c r="G9" s="16" t="s">
-        <v>1152</v>
+        <v>1135</v>
       </c>
       <c r="H9" s="16" t="s">
-        <v>1153</v>
+        <v>1136</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="13" t="s">
-        <v>1154</v>
+        <v>1137</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>1155</v>
+        <v>1138</v>
       </c>
       <c r="C10" s="13"/>
       <c r="D10" s="13"/>
@@ -11171,16 +11171,16 @@
     </row>
     <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
-        <v>1154</v>
+        <v>1137</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>1155</v>
+        <v>1138</v>
       </c>
       <c r="C11" s="15" t="s">
-        <v>1156</v>
+        <v>1139</v>
       </c>
       <c r="D11" s="16" t="s">
-        <v>1157</v>
+        <v>1140</v>
       </c>
       <c r="E11" s="17">
         <v>2</v>
@@ -11189,24 +11189,24 @@
         <v>418</v>
       </c>
       <c r="G11" s="16" t="s">
-        <v>1158</v>
+        <v>1141</v>
       </c>
       <c r="H11" s="16" t="s">
-        <v>1159</v>
+        <v>1142</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="19" t="s">
-        <v>1154</v>
+        <v>1137</v>
       </c>
       <c r="B12" s="19" t="s">
-        <v>1155</v>
+        <v>1138</v>
       </c>
       <c r="C12" s="20" t="s">
-        <v>1160</v>
+        <v>1143</v>
       </c>
       <c r="D12" s="21" t="s">
-        <v>1161</v>
+        <v>1144</v>
       </c>
       <c r="E12" s="17">
         <v>2</v>
@@ -11215,70 +11215,70 @@
         <v>418</v>
       </c>
       <c r="G12" s="21" t="s">
-        <v>1162</v>
+        <v>1145</v>
       </c>
       <c r="H12" s="21" t="s">
-        <v>1163</v>
+        <v>1146</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
-        <v>1154</v>
+        <v>1137</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>1155</v>
+        <v>1138</v>
       </c>
       <c r="C13" s="15" t="s">
-        <v>1164</v>
+        <v>1147</v>
       </c>
       <c r="D13" s="16" t="s">
-        <v>1165</v>
+        <v>1148</v>
       </c>
       <c r="E13" s="17">
         <v>2</v>
       </c>
       <c r="F13" s="18" t="s">
-        <v>12</v>
+        <v>710</v>
       </c>
       <c r="G13" s="16" t="s">
-        <v>1166</v>
+        <v>1309</v>
       </c>
       <c r="H13" s="16" t="s">
-        <v>1167</v>
+        <v>1149</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="19" t="s">
-        <v>1154</v>
+        <v>1137</v>
       </c>
       <c r="B14" s="19" t="s">
-        <v>1155</v>
+        <v>1138</v>
       </c>
       <c r="C14" s="20" t="s">
-        <v>1168</v>
+        <v>1150</v>
       </c>
       <c r="D14" s="21" t="s">
-        <v>1169</v>
+        <v>1151</v>
       </c>
       <c r="E14" s="17">
         <v>2</v>
       </c>
       <c r="F14" s="18" t="s">
-        <v>12</v>
+        <v>418</v>
       </c>
       <c r="G14" s="21" t="s">
-        <v>1170</v>
+        <v>1310</v>
       </c>
       <c r="H14" s="21" t="s">
-        <v>1171</v>
+        <v>1152</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="13" t="s">
-        <v>1172</v>
+        <v>1153</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>1173</v>
+        <v>1154</v>
       </c>
       <c r="C15" s="13"/>
       <c r="D15" s="13"/>
@@ -11289,16 +11289,16 @@
     </row>
     <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="14" t="s">
-        <v>1172</v>
+        <v>1153</v>
       </c>
       <c r="B16" s="14" t="s">
-        <v>1173</v>
+        <v>1154</v>
       </c>
       <c r="C16" s="15" t="s">
-        <v>1174</v>
+        <v>1155</v>
       </c>
       <c r="D16" s="16" t="s">
-        <v>1175</v>
+        <v>1156</v>
       </c>
       <c r="E16" s="17">
         <v>2</v>
@@ -11307,24 +11307,24 @@
         <v>418</v>
       </c>
       <c r="G16" s="16" t="s">
-        <v>1176</v>
+        <v>1157</v>
       </c>
       <c r="H16" s="16" t="s">
-        <v>1177</v>
+        <v>1158</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="19" t="s">
-        <v>1172</v>
+        <v>1153</v>
       </c>
       <c r="B17" s="19" t="s">
-        <v>1173</v>
+        <v>1154</v>
       </c>
       <c r="C17" s="20" t="s">
-        <v>1178</v>
+        <v>1159</v>
       </c>
       <c r="D17" s="21" t="s">
-        <v>1179</v>
+        <v>1160</v>
       </c>
       <c r="E17" s="17">
         <v>2</v>
@@ -11333,24 +11333,24 @@
         <v>12</v>
       </c>
       <c r="G17" s="21" t="s">
-        <v>1180</v>
+        <v>1161</v>
       </c>
       <c r="H17" s="21" t="s">
-        <v>1181</v>
+        <v>1162</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="14" t="s">
-        <v>1172</v>
+        <v>1153</v>
       </c>
       <c r="B18" s="14" t="s">
-        <v>1173</v>
+        <v>1154</v>
       </c>
       <c r="C18" s="15" t="s">
-        <v>1182</v>
+        <v>1163</v>
       </c>
       <c r="D18" s="16" t="s">
-        <v>1183</v>
+        <v>1164</v>
       </c>
       <c r="E18" s="17">
         <v>2</v>
@@ -11359,18 +11359,18 @@
         <v>12</v>
       </c>
       <c r="G18" s="16" t="s">
-        <v>1184</v>
+        <v>1165</v>
       </c>
       <c r="H18" s="16" t="s">
-        <v>1185</v>
+        <v>1166</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="13" t="s">
-        <v>1186</v>
+        <v>1167</v>
       </c>
       <c r="B19" s="13" t="s">
-        <v>1187</v>
+        <v>1168</v>
       </c>
       <c r="C19" s="13"/>
       <c r="D19" s="13"/>
@@ -11381,16 +11381,16 @@
     </row>
     <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="14" t="s">
-        <v>1186</v>
+        <v>1167</v>
       </c>
       <c r="B20" s="14" t="s">
-        <v>1187</v>
+        <v>1168</v>
       </c>
       <c r="C20" s="15" t="s">
-        <v>1188</v>
+        <v>1169</v>
       </c>
       <c r="D20" s="16" t="s">
-        <v>1189</v>
+        <v>1170</v>
       </c>
       <c r="E20" s="17">
         <v>2</v>
@@ -11399,50 +11399,50 @@
         <v>418</v>
       </c>
       <c r="G20" s="16" t="s">
-        <v>1190</v>
+        <v>1171</v>
       </c>
       <c r="H20" s="16" t="s">
-        <v>1191</v>
+        <v>1172</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="19" t="s">
-        <v>1186</v>
+        <v>1167</v>
       </c>
       <c r="B21" s="19" t="s">
-        <v>1187</v>
+        <v>1168</v>
       </c>
       <c r="C21" s="20" t="s">
-        <v>1192</v>
+        <v>1173</v>
       </c>
       <c r="D21" s="21" t="s">
-        <v>1193</v>
+        <v>1174</v>
       </c>
       <c r="E21" s="17">
         <v>2</v>
       </c>
       <c r="F21" s="18" t="s">
-        <v>12</v>
+        <v>710</v>
       </c>
       <c r="G21" s="21" t="s">
-        <v>1194</v>
+        <v>1311</v>
       </c>
       <c r="H21" s="21" t="s">
-        <v>1195</v>
+        <v>1175</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="14" t="s">
-        <v>1186</v>
+        <v>1167</v>
       </c>
       <c r="B22" s="14" t="s">
-        <v>1187</v>
+        <v>1168</v>
       </c>
       <c r="C22" s="15" t="s">
-        <v>1196</v>
+        <v>1176</v>
       </c>
       <c r="D22" s="16" t="s">
-        <v>1197</v>
+        <v>1177</v>
       </c>
       <c r="E22" s="17">
         <v>2</v>
@@ -11451,24 +11451,24 @@
         <v>418</v>
       </c>
       <c r="G22" s="16" t="s">
-        <v>1198</v>
+        <v>1178</v>
       </c>
       <c r="H22" s="16" t="s">
-        <v>1199</v>
+        <v>1179</v>
       </c>
     </row>
     <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="19" t="s">
-        <v>1186</v>
+        <v>1167</v>
       </c>
       <c r="B23" s="19" t="s">
-        <v>1187</v>
+        <v>1168</v>
       </c>
       <c r="C23" s="20" t="s">
-        <v>1200</v>
+        <v>1180</v>
       </c>
       <c r="D23" s="21" t="s">
-        <v>1201</v>
+        <v>1181</v>
       </c>
       <c r="E23" s="23">
         <v>3</v>
@@ -11477,10 +11477,10 @@
         <v>418</v>
       </c>
       <c r="G23" s="21" t="s">
-        <v>1202</v>
+        <v>1182</v>
       </c>
       <c r="H23" s="21" t="s">
-        <v>1199</v>
+        <v>1179</v>
       </c>
     </row>
   </sheetData>
@@ -11549,10 +11549,10 @@
     </row>
     <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
-        <v>1203</v>
+        <v>1183</v>
       </c>
       <c r="B2" s="13" t="s">
-        <v>1204</v>
+        <v>1184</v>
       </c>
       <c r="C2" s="13"/>
       <c r="D2" s="13"/>
@@ -11563,16 +11563,16 @@
     </row>
     <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
-        <v>1203</v>
+        <v>1183</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>1204</v>
+        <v>1184</v>
       </c>
       <c r="C3" s="15" t="s">
-        <v>1205</v>
+        <v>1185</v>
       </c>
       <c r="D3" s="16" t="s">
-        <v>1206</v>
+        <v>1186</v>
       </c>
       <c r="E3" s="17">
         <v>2</v>
@@ -11581,22 +11581,22 @@
         <v>20</v>
       </c>
       <c r="G3" s="16" t="s">
-        <v>1207</v>
+        <v>1187</v>
       </c>
       <c r="H3" s="16"/>
     </row>
     <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="19" t="s">
-        <v>1203</v>
+        <v>1183</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>1204</v>
+        <v>1184</v>
       </c>
       <c r="C4" s="20" t="s">
-        <v>1208</v>
+        <v>1188</v>
       </c>
       <c r="D4" s="21" t="s">
-        <v>1209</v>
+        <v>1189</v>
       </c>
       <c r="E4" s="23">
         <v>3</v>
@@ -11605,16 +11605,16 @@
         <v>20</v>
       </c>
       <c r="G4" s="21" t="s">
-        <v>1210</v>
+        <v>1190</v>
       </c>
       <c r="H4" s="21"/>
     </row>
     <row r="5" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="13" t="s">
-        <v>1211</v>
+        <v>1191</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>1212</v>
+        <v>1192</v>
       </c>
       <c r="C5" s="13"/>
       <c r="D5" s="13"/>
@@ -11625,16 +11625,16 @@
     </row>
     <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>1211</v>
+        <v>1191</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>1212</v>
+        <v>1192</v>
       </c>
       <c r="C6" s="15" t="s">
-        <v>1213</v>
+        <v>1193</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>1214</v>
+        <v>1194</v>
       </c>
       <c r="E6" s="17">
         <v>2</v>
@@ -11643,22 +11643,22 @@
         <v>20</v>
       </c>
       <c r="G6" s="16" t="s">
-        <v>1215</v>
+        <v>1195</v>
       </c>
       <c r="H6" s="16"/>
     </row>
     <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="19" t="s">
-        <v>1211</v>
+        <v>1191</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>1212</v>
+        <v>1192</v>
       </c>
       <c r="C7" s="20" t="s">
-        <v>1216</v>
+        <v>1196</v>
       </c>
       <c r="D7" s="21" t="s">
-        <v>1217</v>
+        <v>1197</v>
       </c>
       <c r="E7" s="17">
         <v>2</v>
@@ -11667,22 +11667,22 @@
         <v>20</v>
       </c>
       <c r="G7" s="21" t="s">
-        <v>1218</v>
+        <v>1198</v>
       </c>
       <c r="H7" s="21"/>
     </row>
     <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
-        <v>1211</v>
+        <v>1191</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>1212</v>
+        <v>1192</v>
       </c>
       <c r="C8" s="15" t="s">
-        <v>1219</v>
+        <v>1199</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>1220</v>
+        <v>1200</v>
       </c>
       <c r="E8" s="17">
         <v>2</v>
@@ -11691,22 +11691,22 @@
         <v>20</v>
       </c>
       <c r="G8" s="16" t="s">
-        <v>1221</v>
+        <v>1201</v>
       </c>
       <c r="H8" s="16"/>
     </row>
     <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="19" t="s">
-        <v>1211</v>
+        <v>1191</v>
       </c>
       <c r="B9" s="19" t="s">
-        <v>1212</v>
+        <v>1192</v>
       </c>
       <c r="C9" s="20" t="s">
-        <v>1222</v>
+        <v>1202</v>
       </c>
       <c r="D9" s="21" t="s">
-        <v>1223</v>
+        <v>1203</v>
       </c>
       <c r="E9" s="17">
         <v>2</v>
@@ -11715,22 +11715,22 @@
         <v>20</v>
       </c>
       <c r="G9" s="21" t="s">
-        <v>1218</v>
+        <v>1198</v>
       </c>
       <c r="H9" s="21"/>
     </row>
     <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
-        <v>1211</v>
+        <v>1191</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>1212</v>
+        <v>1192</v>
       </c>
       <c r="C10" s="15" t="s">
-        <v>1224</v>
+        <v>1204</v>
       </c>
       <c r="D10" s="16" t="s">
-        <v>1225</v>
+        <v>1205</v>
       </c>
       <c r="E10" s="23">
         <v>3</v>
@@ -11739,22 +11739,22 @@
         <v>20</v>
       </c>
       <c r="G10" s="16" t="s">
-        <v>1218</v>
+        <v>1198</v>
       </c>
       <c r="H10" s="16"/>
     </row>
     <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="19" t="s">
-        <v>1211</v>
+        <v>1191</v>
       </c>
       <c r="B11" s="19" t="s">
-        <v>1212</v>
+        <v>1192</v>
       </c>
       <c r="C11" s="20" t="s">
-        <v>1226</v>
+        <v>1206</v>
       </c>
       <c r="D11" s="21" t="s">
-        <v>1227</v>
+        <v>1207</v>
       </c>
       <c r="E11" s="23">
         <v>3</v>
@@ -11763,22 +11763,22 @@
         <v>20</v>
       </c>
       <c r="G11" s="21" t="s">
-        <v>1218</v>
+        <v>1198</v>
       </c>
       <c r="H11" s="21"/>
     </row>
     <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
-        <v>1211</v>
+        <v>1191</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>1212</v>
+        <v>1192</v>
       </c>
       <c r="C12" s="15" t="s">
-        <v>1228</v>
+        <v>1208</v>
       </c>
       <c r="D12" s="16" t="s">
-        <v>1229</v>
+        <v>1209</v>
       </c>
       <c r="E12" s="23">
         <v>3</v>
@@ -11787,22 +11787,22 @@
         <v>20</v>
       </c>
       <c r="G12" s="16" t="s">
-        <v>1230</v>
+        <v>1210</v>
       </c>
       <c r="H12" s="16"/>
     </row>
     <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="19" t="s">
+        <v>1191</v>
+      </c>
+      <c r="B13" s="19" t="s">
+        <v>1192</v>
+      </c>
+      <c r="C13" s="20" t="s">
         <v>1211</v>
       </c>
-      <c r="B13" s="19" t="s">
+      <c r="D13" s="21" t="s">
         <v>1212</v>
-      </c>
-      <c r="C13" s="20" t="s">
-        <v>1231</v>
-      </c>
-      <c r="D13" s="21" t="s">
-        <v>1232</v>
       </c>
       <c r="E13" s="23">
         <v>3</v>
@@ -11811,16 +11811,16 @@
         <v>20</v>
       </c>
       <c r="G13" s="21" t="s">
-        <v>1233</v>
+        <v>1213</v>
       </c>
       <c r="H13" s="21"/>
     </row>
     <row r="14" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="13" t="s">
-        <v>1234</v>
+        <v>1214</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>1235</v>
+        <v>1215</v>
       </c>
       <c r="C14" s="13"/>
       <c r="D14" s="13"/>
@@ -11831,16 +11831,16 @@
     </row>
     <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="14" t="s">
-        <v>1234</v>
+        <v>1214</v>
       </c>
       <c r="B15" s="14" t="s">
-        <v>1235</v>
+        <v>1215</v>
       </c>
       <c r="C15" s="15" t="s">
-        <v>1236</v>
+        <v>1216</v>
       </c>
       <c r="D15" s="16" t="s">
-        <v>1237</v>
+        <v>1217</v>
       </c>
       <c r="E15" s="17">
         <v>2</v>
@@ -11849,22 +11849,22 @@
         <v>20</v>
       </c>
       <c r="G15" s="16" t="s">
-        <v>1238</v>
+        <v>1218</v>
       </c>
       <c r="H15" s="16"/>
     </row>
     <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="19" t="s">
-        <v>1234</v>
+        <v>1214</v>
       </c>
       <c r="B16" s="19" t="s">
-        <v>1235</v>
+        <v>1215</v>
       </c>
       <c r="C16" s="20" t="s">
-        <v>1239</v>
+        <v>1219</v>
       </c>
       <c r="D16" s="21" t="s">
-        <v>1240</v>
+        <v>1220</v>
       </c>
       <c r="E16" s="17">
         <v>2</v>
@@ -11873,7 +11873,7 @@
         <v>20</v>
       </c>
       <c r="G16" s="21" t="s">
-        <v>1238</v>
+        <v>1218</v>
       </c>
       <c r="H16" s="21"/>
     </row>
@@ -12113,7 +12113,7 @@
         <v>418</v>
       </c>
       <c r="G9" s="24" t="s">
-        <v>1241</v>
+        <v>1221</v>
       </c>
       <c r="H9" s="24" t="s">
         <v>141</v>
@@ -12139,7 +12139,7 @@
         <v>20</v>
       </c>
       <c r="G10" s="24" t="s">
-        <v>1242</v>
+        <v>1222</v>
       </c>
       <c r="H10" s="24" t="s">
         <v>144</v>
@@ -12576,7 +12576,7 @@
         <v>418</v>
       </c>
       <c r="G28" s="24" t="s">
-        <v>1243</v>
+        <v>1223</v>
       </c>
       <c r="H28" s="24" t="s">
         <v>157</v>
@@ -12856,7 +12856,7 @@
         <v>710</v>
       </c>
       <c r="G3" s="24" t="s">
-        <v>1250</v>
+        <v>1230</v>
       </c>
       <c r="H3" s="24" t="s">
         <v>210</v>
@@ -12882,7 +12882,7 @@
         <v>710</v>
       </c>
       <c r="G4" s="24" t="s">
-        <v>1251</v>
+        <v>1231</v>
       </c>
       <c r="H4" s="24" t="s">
         <v>232</v>
@@ -12908,7 +12908,7 @@
         <v>710</v>
       </c>
       <c r="G5" s="24" t="s">
-        <v>1252</v>
+        <v>1232</v>
       </c>
       <c r="H5" s="24" t="s">
         <v>235</v>
@@ -12948,7 +12948,7 @@
         <v>418</v>
       </c>
       <c r="G7" s="24" t="s">
-        <v>1244</v>
+        <v>1224</v>
       </c>
       <c r="H7" s="24" t="s">
         <v>210</v>
@@ -12974,7 +12974,7 @@
         <v>418</v>
       </c>
       <c r="G8" s="24" t="s">
-        <v>1245</v>
+        <v>1225</v>
       </c>
       <c r="H8" s="24" t="s">
         <v>242</v>
@@ -13000,7 +13000,7 @@
         <v>418</v>
       </c>
       <c r="G9" s="24" t="s">
-        <v>1246</v>
+        <v>1226</v>
       </c>
       <c r="H9" s="24" t="s">
         <v>245</v>
@@ -13066,7 +13066,7 @@
         <v>710</v>
       </c>
       <c r="G12" s="24" t="s">
-        <v>1248</v>
+        <v>1228</v>
       </c>
       <c r="H12" s="24" t="s">
         <v>254</v>
@@ -13092,7 +13092,7 @@
         <v>418</v>
       </c>
       <c r="G13" s="24" t="s">
-        <v>1247</v>
+        <v>1227</v>
       </c>
       <c r="H13" s="24" t="s">
         <v>257</v>
@@ -13182,7 +13182,7 @@
         <v>710</v>
       </c>
       <c r="G17" s="24" t="s">
-        <v>1249</v>
+        <v>1229</v>
       </c>
       <c r="H17" s="24" t="s">
         <v>268</v>
@@ -13570,7 +13570,7 @@
         <v>418</v>
       </c>
       <c r="G15" s="24" t="s">
-        <v>1253</v>
+        <v>1233</v>
       </c>
       <c r="H15" s="16"/>
     </row>
@@ -13594,7 +13594,7 @@
         <v>418</v>
       </c>
       <c r="G16" s="24" t="s">
-        <v>1254</v>
+        <v>1234</v>
       </c>
       <c r="H16" s="21"/>
     </row>
@@ -13642,7 +13642,7 @@
         <v>418</v>
       </c>
       <c r="G18" s="21" t="s">
-        <v>1255</v>
+        <v>1235</v>
       </c>
       <c r="H18" s="21"/>
     </row>
@@ -13776,7 +13776,7 @@
         <v>418</v>
       </c>
       <c r="G24" s="16" t="s">
-        <v>1256</v>
+        <v>1236</v>
       </c>
       <c r="H24" s="16"/>
     </row>
@@ -13800,7 +13800,7 @@
         <v>20</v>
       </c>
       <c r="G25" s="21" t="s">
-        <v>1257</v>
+        <v>1237</v>
       </c>
       <c r="H25" s="21"/>
     </row>
@@ -13824,7 +13824,7 @@
         <v>418</v>
       </c>
       <c r="G26" s="16" t="s">
-        <v>1258</v>
+        <v>1238</v>
       </c>
       <c r="H26" s="16"/>
     </row>
@@ -14218,7 +14218,7 @@
         <v>418</v>
       </c>
       <c r="G3" s="16" t="s">
-        <v>1259</v>
+        <v>1239</v>
       </c>
       <c r="H3" s="16"/>
     </row>
@@ -14266,7 +14266,7 @@
         <v>710</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>1260</v>
+        <v>1240</v>
       </c>
       <c r="H5" s="16"/>
     </row>
@@ -14290,7 +14290,7 @@
         <v>418</v>
       </c>
       <c r="G6" s="21" t="s">
-        <v>1261</v>
+        <v>1241</v>
       </c>
       <c r="H6" s="21"/>
     </row>
@@ -14352,7 +14352,7 @@
         <v>418</v>
       </c>
       <c r="G9" s="16" t="s">
-        <v>1262</v>
+        <v>1242</v>
       </c>
       <c r="H9" s="16"/>
     </row>
@@ -14376,7 +14376,7 @@
         <v>418</v>
       </c>
       <c r="G10" s="21" t="s">
-        <v>1263</v>
+        <v>1243</v>
       </c>
       <c r="H10" s="21"/>
     </row>
@@ -14400,7 +14400,7 @@
         <v>418</v>
       </c>
       <c r="G11" s="16" t="s">
-        <v>1264</v>
+        <v>1244</v>
       </c>
       <c r="H11" s="16"/>
     </row>
@@ -14424,7 +14424,7 @@
         <v>418</v>
       </c>
       <c r="G12" s="21" t="s">
-        <v>1265</v>
+        <v>1245</v>
       </c>
       <c r="H12" s="21"/>
     </row>
@@ -14448,7 +14448,7 @@
         <v>418</v>
       </c>
       <c r="G13" s="16" t="s">
-        <v>1266</v>
+        <v>1246</v>
       </c>
       <c r="H13" s="16"/>
     </row>
@@ -14920,7 +14920,7 @@
         <v>418</v>
       </c>
       <c r="G12" s="16" t="s">
-        <v>1267</v>
+        <v>1247</v>
       </c>
       <c r="H12" s="16" t="s">
         <v>442</v>
@@ -15036,7 +15036,7 @@
         <v>20</v>
       </c>
       <c r="G17" s="21" t="s">
-        <v>1268</v>
+        <v>1248</v>
       </c>
       <c r="H17" s="21" t="s">
         <v>157</v>
@@ -15164,7 +15164,7 @@
         <v>418</v>
       </c>
       <c r="G3" s="16" t="s">
-        <v>1269</v>
+        <v>1249</v>
       </c>
       <c r="H3" s="16" t="s">
         <v>464</v>
@@ -15280,7 +15280,7 @@
         <v>418</v>
       </c>
       <c r="G8" s="21" t="s">
-        <v>1270</v>
+        <v>1250</v>
       </c>
       <c r="H8" s="21" t="s">
         <v>480</v>
@@ -15358,7 +15358,7 @@
         <v>418</v>
       </c>
       <c r="G11" s="16" t="s">
-        <v>1271</v>
+        <v>1251</v>
       </c>
       <c r="H11" s="16" t="s">
         <v>468</v>
@@ -15484,7 +15484,7 @@
         <v>418</v>
       </c>
       <c r="G16" s="21" t="s">
-        <v>1272</v>
+        <v>1252</v>
       </c>
       <c r="H16" s="21" t="s">
         <v>468</v>
@@ -15536,7 +15536,7 @@
         <v>418</v>
       </c>
       <c r="G18" s="21" t="s">
-        <v>1273</v>
+        <v>1253</v>
       </c>
       <c r="H18" s="21" t="s">
         <v>468</v>
@@ -15652,7 +15652,7 @@
         <v>418</v>
       </c>
       <c r="G23" s="21" t="s">
-        <v>1274</v>
+        <v>1254</v>
       </c>
       <c r="H23" s="21" t="s">
         <v>29</v>
@@ -15794,7 +15794,7 @@
         <v>20</v>
       </c>
       <c r="G29" s="16" t="s">
-        <v>1275</v>
+        <v>1255</v>
       </c>
       <c r="H29" s="16" t="s">
         <v>544</v>
@@ -16510,7 +16510,7 @@
         <v>418</v>
       </c>
       <c r="G3" s="16" t="s">
-        <v>1276</v>
+        <v>1256</v>
       </c>
       <c r="H3" s="16" t="s">
         <v>621</v>
@@ -16600,7 +16600,7 @@
         <v>418</v>
       </c>
       <c r="G7" s="16" t="s">
-        <v>1277</v>
+        <v>1257</v>
       </c>
       <c r="H7" s="16" t="s">
         <v>633</v>
@@ -16626,7 +16626,7 @@
         <v>418</v>
       </c>
       <c r="G8" s="21" t="s">
-        <v>1278</v>
+        <v>1258</v>
       </c>
       <c r="H8" s="21" t="s">
         <v>29</v>
@@ -16676,7 +16676,7 @@
         <v>710</v>
       </c>
       <c r="G10" s="21" t="s">
-        <v>1279</v>
+        <v>1259</v>
       </c>
       <c r="H10" s="21" t="s">
         <v>29</v>
@@ -17168,7 +17168,7 @@
         <v>710</v>
       </c>
       <c r="G4" s="21" t="s">
-        <v>1280</v>
+        <v>1260</v>
       </c>
       <c r="H4" s="21" t="s">
         <v>699</v>
@@ -17282,7 +17282,7 @@
         <v>418</v>
       </c>
       <c r="G9" s="21" t="s">
-        <v>1281</v>
+        <v>1261</v>
       </c>
       <c r="H9" s="21" t="s">
         <v>715</v>
@@ -17308,7 +17308,7 @@
         <v>418</v>
       </c>
       <c r="G10" s="16" t="s">
-        <v>1282</v>
+        <v>1262</v>
       </c>
       <c r="H10" s="16" t="s">
         <v>718</v>
@@ -17372,7 +17372,7 @@
         <v>418</v>
       </c>
       <c r="G13" s="16" t="s">
-        <v>1283</v>
+        <v>1263</v>
       </c>
       <c r="H13" s="16" t="s">
         <v>726</v>
@@ -17398,7 +17398,7 @@
         <v>710</v>
       </c>
       <c r="G14" s="21" t="s">
-        <v>1284</v>
+        <v>1264</v>
       </c>
       <c r="H14" s="21" t="s">
         <v>729</v>
@@ -17424,7 +17424,7 @@
         <v>418</v>
       </c>
       <c r="G15" s="16" t="s">
-        <v>1285</v>
+        <v>1265</v>
       </c>
       <c r="H15" s="16" t="s">
         <v>732</v>

</xml_diff>